<commit_message>
feat(config): G03-P3-B5 author universe rules and evidence
</commit_message>
<xml_diff>
--- a/config/generated/templates/UniverseBindings.xlsx
+++ b/config/generated/templates/UniverseBindings.xlsx
@@ -987,8 +987,8 @@
       <formula1>1</formula1>
       <formula2>2147483647</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Blessing, Curio, Occurrence, Encounter, Shop" promptTitle="UniversePoolKind enum" prompt="Select a value from the dropdown." sqref="D8:D1007">
-      <formula1>"Blessing,Curio,Occurrence,Encounter,Shop"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid enum value" error="Value must be one of: Blessing, Curio, Occurrence, Encounter, Shop, TrailblazeBonus" promptTitle="UniversePoolKind enum" prompt="Select a value from the dropdown." sqref="D8:D1007">
+      <formula1>"Blessing,Curio,Occurrence,Encounter,Shop,TrailblazeBonus"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid boolean value" error="Value must be true or false." promptTitle="Boolean" prompt="Select true or false." sqref="F8:F1007">
       <formula1>"true,false"</formula1>

</xml_diff>